<commit_message>
data updated (email id)
</commit_message>
<xml_diff>
--- a/Notification/data/raw/contact_details.xlsx
+++ b/Notification/data/raw/contact_details.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Tanmay\End Sem PBL\testing_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Tanmay\End Sem PBL\end-sem-practical-pbl\Notification\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A655889-5A56-48B4-A196-25B105FD97CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77CFAA97-23F0-4EAC-BC92-26769492F219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{24530F12-58D8-4835-8E6E-93F1C2567B79}"/>
   </bookViews>
@@ -81,7 +81,7 @@
     <t>whatsapp</t>
   </si>
   <si>
-    <t>tanmayjain@gmail.com</t>
+    <t>tanmaysspu@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -649,7 +649,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{E5BFC112-DEAC-426A-84EC-D2C56E3DAE5C}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{195936EC-6050-4830-BAB6-8D06446FB56C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>